<commit_message>
fix: student and staff import mapping, added mother/emergency mobile fields
</commit_message>
<xml_diff>
--- a/Students_Import_Template.xlsx
+++ b/Students_Import_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sms\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{890214F9-0E0E-4664-9A6D-5CDC896B1D9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCFDBA81-003B-4046-A0EC-A293F489BFA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,18 @@
     <sheet name="Student Data" sheetId="1" r:id="rId1"/>
     <sheet name="Instructions" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -143,9 +154,6 @@
     <t>Muhammad Zohan Fareed</t>
   </si>
   <si>
-    <t>mubariz Hassan</t>
-  </si>
-  <si>
     <t>M.Taha</t>
   </si>
   <si>
@@ -155,21 +163,9 @@
     <t>Tabiah Tauqir</t>
   </si>
   <si>
-    <t>umaima</t>
-  </si>
-  <si>
-    <t>zunaisha</t>
-  </si>
-  <si>
-    <t>rania Hashmi</t>
-  </si>
-  <si>
     <t>Shahmeer Raza</t>
   </si>
   <si>
-    <t>Umm e HAni</t>
-  </si>
-  <si>
     <t>Hajra Bibi</t>
   </si>
   <si>
@@ -197,21 +193,12 @@
     <t>Syed Arham Areeb</t>
   </si>
   <si>
-    <t>abdul samad</t>
-  </si>
-  <si>
     <t>Muhammad Subayyal Abdullah</t>
   </si>
   <si>
     <t>Haya Fatima</t>
   </si>
   <si>
-    <t>HASSAN RAZZAQ</t>
-  </si>
-  <si>
-    <t>HAIDER FURQAN</t>
-  </si>
-  <si>
     <t>Farid Ahmed Javed</t>
   </si>
   <si>
@@ -227,18 +214,9 @@
     <t>Hafiz Muhammad Tauqir Irshad</t>
   </si>
   <si>
-    <t>M. zafran</t>
-  </si>
-  <si>
-    <t>waqas anwar</t>
-  </si>
-  <si>
     <t>Abdul Rasheed</t>
   </si>
   <si>
-    <t>ALI RAZA SYED</t>
-  </si>
-  <si>
     <t>M. Abbas</t>
   </si>
   <si>
@@ -251,9 +229,6 @@
     <t>Khuram Javed</t>
   </si>
   <si>
-    <t>javaid Iqbal</t>
-  </si>
-  <si>
     <t>Ahsen Mukhtar</t>
   </si>
   <si>
@@ -269,19 +244,55 @@
     <t>Syed Areeb Bari</t>
   </si>
   <si>
-    <t>muhammad faheem</t>
-  </si>
-  <si>
-    <t>muhammad</t>
-  </si>
-  <si>
     <t>Danish Ishaq</t>
   </si>
   <si>
-    <t>ADNAN RAZZAQ</t>
-  </si>
-  <si>
-    <t>FURQAN SHABIR</t>
+    <t>Mubariz Hassan</t>
+  </si>
+  <si>
+    <t>Umaima</t>
+  </si>
+  <si>
+    <t>Zunaisha</t>
+  </si>
+  <si>
+    <t>Rania Hashmi</t>
+  </si>
+  <si>
+    <t>Umm E Hani</t>
+  </si>
+  <si>
+    <t>Abdul Samad</t>
+  </si>
+  <si>
+    <t>Hassan Razzaq</t>
+  </si>
+  <si>
+    <t>Haider Furqan</t>
+  </si>
+  <si>
+    <t>M. Zafran</t>
+  </si>
+  <si>
+    <t>Waqas Anwar</t>
+  </si>
+  <si>
+    <t>Ali Raza Syed</t>
+  </si>
+  <si>
+    <t>Javaid Iqbal</t>
+  </si>
+  <si>
+    <t>Muhammad Faheem</t>
+  </si>
+  <si>
+    <t>Muhammad</t>
+  </si>
+  <si>
+    <t>Adnan Razzaq</t>
+  </si>
+  <si>
+    <t>Furqan Shabir</t>
   </si>
 </sst>
 </file>
@@ -735,7 +746,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D2" s="2">
         <v>3217579313</v>
@@ -746,13 +757,13 @@
     </row>
     <row r="3" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
       <c r="D3" s="2">
         <v>3007014219</v>
@@ -763,13 +774,13 @@
     </row>
     <row r="4" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="D4" s="2">
         <v>3009611262</v>
@@ -780,13 +791,13 @@
     </row>
     <row r="5" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B5" s="1">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="D5" s="2">
         <v>3216829995</v>
@@ -797,13 +808,13 @@
     </row>
     <row r="6" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B6" s="1">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="D6" s="2">
         <v>3458730300</v>
@@ -814,13 +825,13 @@
     </row>
     <row r="7" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="B7" s="1">
         <v>6</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="D7" s="2">
         <v>3276163490</v>
@@ -831,13 +842,13 @@
     </row>
     <row r="8" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="B8" s="1">
         <v>7</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>69</v>
+        <v>80</v>
       </c>
       <c r="D8" s="2">
         <v>3049356676</v>
@@ -848,13 +859,13 @@
     </row>
     <row r="9" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>46</v>
+        <v>74</v>
       </c>
       <c r="B9" s="1">
         <v>8</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="D9" s="2">
         <v>3136930930</v>
@@ -865,13 +876,13 @@
     </row>
     <row r="10" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="D10" s="2">
         <v>3000789211</v>
@@ -882,13 +893,13 @@
     </row>
     <row r="11" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>48</v>
+        <v>75</v>
       </c>
       <c r="B11" s="1">
         <v>10</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="D11" s="2">
         <v>3007014219</v>
@@ -899,13 +910,13 @@
     </row>
     <row r="12" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B12" s="1">
         <v>11</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>73</v>
+        <v>62</v>
       </c>
       <c r="D12" s="2">
         <v>3017704236</v>
@@ -916,13 +927,13 @@
     </row>
     <row r="13" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B13" s="1">
         <v>12</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="D13" s="2">
         <v>3029408466</v>
@@ -933,13 +944,13 @@
     </row>
     <row r="14" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B14" s="1">
         <v>13</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="D14" s="2">
         <v>3458704060</v>
@@ -950,13 +961,13 @@
     </row>
     <row r="15" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B15" s="1">
         <v>14</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="D15" s="2">
         <v>3280218603</v>
@@ -967,13 +978,13 @@
     </row>
     <row r="16" spans="1:10" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B16" s="1">
         <v>15</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="D16" s="2">
         <v>3002650003</v>
@@ -984,13 +995,13 @@
     </row>
     <row r="17" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B17" s="1">
         <v>16</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="D17" s="2">
         <v>3006855586</v>
@@ -1001,13 +1012,13 @@
     </row>
     <row r="18" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B18" s="1">
         <v>17</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="D18" s="2">
         <v>3022563345</v>
@@ -1018,13 +1029,13 @@
     </row>
     <row r="19" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B19" s="1">
         <v>18</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="D19" s="2">
         <v>3365025803</v>
@@ -1035,13 +1046,13 @@
     </row>
     <row r="20" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B20" s="1">
         <v>19</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="D20" s="2">
         <v>3111001800</v>
@@ -1052,13 +1063,13 @@
     </row>
     <row r="21" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="B21" s="1">
         <v>20</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D21" s="2">
         <v>3023605351</v>
@@ -1069,13 +1080,13 @@
     </row>
     <row r="22" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B22" s="1">
         <v>21</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D22" s="2">
         <v>3006892610</v>
@@ -1086,13 +1097,13 @@
     </row>
     <row r="23" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="B23" s="1">
         <v>22</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="D23" s="2">
         <v>3106819009</v>
@@ -1103,7 +1114,7 @@
     </row>
     <row r="24" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="B24" s="1">
         <v>23</v>
@@ -1120,7 +1131,7 @@
     </row>
     <row r="25" spans="1:7" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B25" s="1">
         <v>24</v>

</xml_diff>